<commit_message>
feat(casB_C): Testing and done
Compare runpf, runopf vs model
</commit_message>
<xml_diff>
--- a/01_Data/03_Test_Cases/caso_IEEE6_ww_A.xlsx
+++ b/01_Data/03_Test_Cases/caso_IEEE6_ww_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\2. Universidad Nacional de Colombia\2. Postgraduate\1_SEMESTER\TESIS DE MAESTRIA\2nd Search\04_TESIS_DANIEL\03_CODIGO_TRABAJO_DANIEL\BESS_FACTS_master\01_Data\03_Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613D0DC1-4FE0-44EB-BE66-B2079DDDC34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E797052F-8618-4DF4-865D-AB6BB5BA423C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1806,7 +1806,7 @@
         <v>50</v>
       </c>
       <c r="E6" s="5">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F6" s="9">
         <v>200</v>
@@ -1847,7 +1847,7 @@
         <v>37.5</v>
       </c>
       <c r="E7" s="5">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F7" s="9">
         <v>150</v>

</xml_diff>